<commit_message>
Update talks since starting
</commit_message>
<xml_diff>
--- a/past_talks/TalksSinceIStarted.xlsx
+++ b/past_talks/TalksSinceIStarted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11110"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mapyh/Documents/own-code/maaretp-site/past_talks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maaretp/Documents/own-code/maaretp-site/past_talks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040042E3-6EF1-F84F-B3A9-62C3DB4158E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40736427-7F86-4E4F-B1F3-726B34ED6343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="760" windowWidth="30200" windowHeight="19980" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Talks" sheetId="1" r:id="rId1"/>
@@ -196,7 +196,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -212,6 +212,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -238,7 +239,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -315,10 +316,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Talks!$A$3:$A$25</c:f>
+              <c:f>Talks!$A$3:$A$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
                   <c:v>2001</c:v>
                 </c:pt>
@@ -387,16 +388,19 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2024</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Talks!$B$3:$B$25</c:f>
+              <c:f>Talks!$B$3:$B$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
                   <c:v>5</c:v>
                 </c:pt>
@@ -465,6 +469,9 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>18</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -539,7 +546,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -565,7 +572,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> over time (Total: 529)</a:t>
+              <a:t> over time (Total: 547)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -688,10 +695,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Talks!$C$3:$C$25</c:f>
+              <c:f>Talks!$C$3:$C$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
                   <c:v>5</c:v>
                 </c:pt>
@@ -760,6 +767,9 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>16</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -865,10 +875,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Talks!$G$3:$G$25</c:f>
+              <c:f>Talks!$G$3:$G$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -937,6 +947,9 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1042,10 +1055,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Talks!$K$3:$K$25</c:f>
+              <c:f>Talks!$K$3:$K$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="23"/>
+                <c:ptCount val="24"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1114,6 +1127,9 @@
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1193,7 +1209,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1249,7 +1265,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-FI"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2178,7 +2194,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-FI"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="669579232"/>
@@ -2233,7 +2249,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-FI"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="669839264"/>
@@ -2281,7 +2297,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-FI"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2813,7 +2829,7 @@
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>622300</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3241,7 +3257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="6" width="10.83203125" customWidth="1"/>
@@ -3768,10 +3784,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B27">
-        <f>SUM(B3:B25)</f>
-        <v>529</v>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>2024</v>
+      </c>
+      <c r="B26">
+        <v>18</v>
+      </c>
+      <c r="C26" s="11">
+        <v>16</v>
+      </c>
+      <c r="G26" s="11">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <f>SUM(B3:B26)</f>
+        <v>547</v>
       </c>
     </row>
   </sheetData>
@@ -4871,4 +4904,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d9290083-bd2f-48a2-8ac5-09a524b17d15}" enabled="1" method="Privileged" siteId="{b9fec68c-c92d-461e-9a97-3d03a0f18b82}" contentBits="1" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Update brochures and stats
</commit_message>
<xml_diff>
--- a/past_talks/TalksSinceIStarted.xlsx
+++ b/past_talks/TalksSinceIStarted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maaretp/Documents/own-code/maaretp-site/past_talks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40736427-7F86-4E4F-B1F3-726B34ED6343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BF5852-33DE-5948-B19C-A0537CEA9297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -196,7 +196,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -212,7 +212,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -265,7 +264,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> 529)</a:t>
+              <a:t> 550)</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -462,7 +461,7 @@
                   <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>43</c:v>
+                  <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>39</c:v>
@@ -471,7 +470,7 @@
                   <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -572,7 +571,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> over time (Total: 547)</a:t>
+              <a:t> over time (Total: 550)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -760,7 +759,7 @@
                   <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>9</c:v>
@@ -769,7 +768,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>16</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3733,10 +3732,10 @@
       </c>
       <c r="B23">
         <f>SUM(C23:K23)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C23" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G23" s="3">
         <v>25</v>
@@ -3789,12 +3788,12 @@
         <v>2024</v>
       </c>
       <c r="B26">
-        <v>18</v>
-      </c>
-      <c r="C26" s="11">
-        <v>16</v>
-      </c>
-      <c r="G26" s="11">
+        <v>20</v>
+      </c>
+      <c r="C26" s="3">
+        <v>17</v>
+      </c>
+      <c r="G26" s="3">
         <v>0</v>
       </c>
       <c r="K26">
@@ -3804,7 +3803,7 @@
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28">
         <f>SUM(B3:B26)</f>
-        <v>547</v>
+        <v>550</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add QT panel recording
</commit_message>
<xml_diff>
--- a/past_talks/TalksSinceIStarted.xlsx
+++ b/past_talks/TalksSinceIStarted.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maaretp/Documents/own-code/maaretp-site/past_talks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BF5852-33DE-5948-B19C-A0537CEA9297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C95AAFF-0B7F-D440-AB73-6447F8A89D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -196,7 +196,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -212,6 +212,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -2265,6 +2266,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2272,7 +2274,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2828,7 +2829,7 @@
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>622300</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3256,7 +3257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="6" width="10.83203125" customWidth="1"/>
@@ -3800,8 +3801,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B28">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>2025</v>
+      </c>
+      <c r="C27" s="11"/>
+      <c r="G27" s="11"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B29">
         <f>SUM(B3:B26)</f>
         <v>550</v>
       </c>

</xml_diff>